<commit_message>
Data: Remplacement isic.xlsx par la version mise a jour + regeneration students_clean.csv
</commit_message>
<xml_diff>
--- a/data/raw/isic.xlsx
+++ b/data/raw/isic.xlsx
@@ -1009,7 +1009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Z40"/>
+  <dimension ref="A1:Z39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="25" min="1" max="1"/>
@@ -4293,7 +4293,6 @@
         </is>
       </c>
     </row>
-    <row r="40"/>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="N2:W2"/>
@@ -4314,7 +4313,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Z40"/>
+  <dimension ref="A1:Z39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="25" min="1" max="1"/>
@@ -7598,7 +7597,6 @@
         </is>
       </c>
     </row>
-    <row r="40"/>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="N2:W2"/>
@@ -7619,7 +7617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P39"/>
+  <dimension ref="A1:P35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="26" min="1" max="1"/>
@@ -8751,126 +8749,10 @@
       <c r="O35" s="76" t="n"/>
       <c r="P35" s="69" t="n"/>
     </row>
-    <row r="36" ht="18" customHeight="1" s="26">
-      <c r="A36" s="77" t="inlineStr">
-        <is>
-          <t>M399693</t>
-        </is>
-      </c>
-      <c r="B36" s="77" t="inlineStr">
-        <is>
-          <t>Fassi</t>
-        </is>
-      </c>
-      <c r="C36" s="77" t="inlineStr">
-        <is>
-          <t>Soukaina</t>
-        </is>
-      </c>
-      <c r="D36" s="73" t="n"/>
-      <c r="E36" s="65" t="n"/>
-      <c r="F36" s="65" t="n"/>
-      <c r="G36" s="65" t="n"/>
-      <c r="H36" s="65" t="n"/>
-      <c r="I36" s="65" t="n"/>
-      <c r="J36" s="65" t="n"/>
-      <c r="K36" s="65" t="n"/>
-      <c r="L36" s="74" t="n"/>
-      <c r="M36" s="66" t="n"/>
-      <c r="N36" s="75" t="n"/>
-      <c r="O36" s="76" t="n"/>
-      <c r="P36" s="69" t="n"/>
-    </row>
-    <row r="37" ht="18" customHeight="1" s="26">
-      <c r="A37" s="63" t="inlineStr">
-        <is>
-          <t>T841665</t>
-        </is>
-      </c>
-      <c r="B37" s="63" t="inlineStr">
-        <is>
-          <t>Ghali</t>
-        </is>
-      </c>
-      <c r="C37" s="63" t="inlineStr">
-        <is>
-          <t>Anas</t>
-        </is>
-      </c>
-      <c r="D37" s="73" t="n"/>
-      <c r="E37" s="65" t="n"/>
-      <c r="F37" s="65" t="n"/>
-      <c r="G37" s="65" t="n"/>
-      <c r="H37" s="65" t="n"/>
-      <c r="I37" s="65" t="n"/>
-      <c r="J37" s="65" t="n"/>
-      <c r="K37" s="65" t="n"/>
-      <c r="L37" s="74" t="n"/>
-      <c r="M37" s="66" t="n"/>
-      <c r="N37" s="75" t="n"/>
-      <c r="O37" s="76" t="n"/>
-      <c r="P37" s="69" t="n"/>
-    </row>
-    <row r="38" ht="18" customHeight="1" s="26">
-      <c r="A38" s="77" t="inlineStr">
-        <is>
-          <t>R555717</t>
-        </is>
-      </c>
-      <c r="B38" s="77" t="inlineStr">
-        <is>
-          <t>Harrak</t>
-        </is>
-      </c>
-      <c r="C38" s="77" t="inlineStr">
-        <is>
-          <t>Zineb</t>
-        </is>
-      </c>
-      <c r="D38" s="73" t="n"/>
-      <c r="E38" s="65" t="n"/>
-      <c r="F38" s="65" t="n"/>
-      <c r="G38" s="65" t="n"/>
-      <c r="H38" s="65" t="n"/>
-      <c r="I38" s="65" t="n"/>
-      <c r="J38" s="65" t="n"/>
-      <c r="K38" s="65" t="n"/>
-      <c r="L38" s="74" t="n"/>
-      <c r="M38" s="66" t="n"/>
-      <c r="N38" s="75" t="n"/>
-      <c r="O38" s="76" t="n"/>
-      <c r="P38" s="69" t="n"/>
-    </row>
-    <row r="39" ht="18" customHeight="1" s="26">
-      <c r="A39" s="63" t="inlineStr">
-        <is>
-          <t>T636960</t>
-        </is>
-      </c>
-      <c r="B39" s="63" t="inlineStr">
-        <is>
-          <t>Idmansour</t>
-        </is>
-      </c>
-      <c r="C39" s="63" t="inlineStr">
-        <is>
-          <t>Nabil</t>
-        </is>
-      </c>
-      <c r="D39" s="73" t="n"/>
-      <c r="E39" s="65" t="n"/>
-      <c r="F39" s="65" t="n"/>
-      <c r="G39" s="65" t="n"/>
-      <c r="H39" s="65" t="n"/>
-      <c r="I39" s="65" t="n"/>
-      <c r="J39" s="65" t="n"/>
-      <c r="K39" s="65" t="n"/>
-      <c r="L39" s="74" t="n"/>
-      <c r="M39" s="66" t="n"/>
-      <c r="N39" s="75" t="n"/>
-      <c r="O39" s="76" t="n"/>
-      <c r="P39" s="69" t="n"/>
-    </row>
+    <row r="36" ht="18" customHeight="1" s="26"/>
+    <row r="37" ht="18" customHeight="1" s="26"/>
+    <row r="38" ht="18" customHeight="1" s="26"/>
+    <row r="39" ht="18" customHeight="1" s="26"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="D2:M2"/>

</xml_diff>